<commit_message>
Mark lots 6-10 as paid
</commit_message>
<xml_diff>
--- a/data/lot-details.xlsx
+++ b/data/lot-details.xlsx
@@ -2069,8 +2069,10 @@
       <c r="U7" s="32" t="n">
         <v>46170</v>
       </c>
-      <c r="V7" s="10" t="n">
-        <v>20</v>
+      <c r="V7" s="10" t="inlineStr">
+        <is>
+          <t>已付</t>
+        </is>
       </c>
       <c r="W7" s="5" t="inlineStr">
         <is>
@@ -2160,7 +2162,11 @@
           <t>5月3日</t>
         </is>
       </c>
-      <c r="V8" s="5" t="n"/>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>已付</t>
+        </is>
+      </c>
       <c r="W8" s="5" t="inlineStr">
         <is>
           <t>已抵上海</t>
@@ -2245,7 +2251,11 @@
       <c r="U9" s="31" t="n">
         <v>46192</v>
       </c>
-      <c r="V9" s="5" t="n"/>
+      <c r="V9" s="5" t="inlineStr">
+        <is>
+          <t>已付</t>
+        </is>
+      </c>
       <c r="W9" s="5" t="inlineStr">
         <is>
           <t>已抵上海</t>
@@ -2334,7 +2344,11 @@
           <t>5月11日</t>
         </is>
       </c>
-      <c r="V10" s="5" t="n"/>
+      <c r="V10" s="5" t="inlineStr">
+        <is>
+          <t>已付</t>
+        </is>
+      </c>
       <c r="W10" s="5" t="inlineStr">
         <is>
           <t>已抵上海</t>
@@ -2423,7 +2437,11 @@
           <t>5月11日</t>
         </is>
       </c>
-      <c r="V11" s="5" t="n"/>
+      <c r="V11" s="5" t="inlineStr">
+        <is>
+          <t>已付</t>
+        </is>
+      </c>
       <c r="W11" s="5" t="inlineStr">
         <is>
           <t>已抵上海</t>
@@ -2512,7 +2530,11 @@
           <t>5月11日</t>
         </is>
       </c>
-      <c r="V12" s="5" t="n"/>
+      <c r="V12" s="5" t="inlineStr">
+        <is>
+          <t>已付</t>
+        </is>
+      </c>
       <c r="W12" s="5" t="inlineStr">
         <is>
           <t>已抵上海</t>

</xml_diff>